<commit_message>
Add judgment rows to samples, tidy README
- samples/*.xlsx: 寸法判定・重量判定・総合判定を各帳票に追加
- output/aggregate_report.xlsx: 再生成
- README.md: generate_samples.py に関する記述を削除、コマンド例を python に統一
</commit_message>
<xml_diff>
--- a/samples/sample_01_A0001.xlsx
+++ b/samples/sample_01_A0001.xlsx
@@ -346,7 +346,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B3:E14"/>
+  <dimension ref="B3:E17"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.63" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col width="4.25" customWidth="1" style="5" min="1" max="1"/>
@@ -446,6 +446,42 @@
         </is>
       </c>
     </row>
+    <row r="15">
+      <c r="B15" s="1" t="inlineStr">
+        <is>
+          <t>寸法判定</t>
+        </is>
+      </c>
+      <c r="C15" s="4" t="inlineStr">
+        <is>
+          <t>合格</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="B16" s="1" t="inlineStr">
+        <is>
+          <t>重量判定</t>
+        </is>
+      </c>
+      <c r="C16" s="4" t="inlineStr">
+        <is>
+          <t>合格</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="B17" s="1" t="inlineStr">
+        <is>
+          <t>総合判定</t>
+        </is>
+      </c>
+      <c r="C17" s="4" t="inlineStr">
+        <is>
+          <t>合格</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>